<commit_message>
Upload current EHR-Predict project state
</commit_message>
<xml_diff>
--- a/data dicision/field adapter/field_explanation_table_v1.xlsx
+++ b/data dicision/field adapter/field_explanation_table_v1.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\vanila\code\EHR-Predict\data dicision\field adapter\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09A9CDB0-16BD-4DBE-BB18-E606F8639A37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="explanation" sheetId="1" r:id="rId1"/>
@@ -13,12 +19,12 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">explanation!$A$1:$G$20</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="162">
   <si>
     <t>group</t>
   </si>
@@ -110,90 +116,96 @@
     <t>G2</t>
   </si>
   <si>
-    <t>age / male</t>
+    <t>age</t>
+  </si>
+  <si>
+    <t>STATIC bucket token</t>
+  </si>
+  <si>
+    <t>patients/admissions</t>
+  </si>
+  <si>
+    <t>6 buckets: 18-39/40-54/55-64/65-74/75-84/85-89. No numeric channel.</t>
+  </si>
+  <si>
+    <t>Admission-known static fields.</t>
+  </si>
+  <si>
+    <t>No temporal leakage.</t>
+  </si>
+  <si>
+    <t>male/mechanism_cat/transfer/head_injury/ed_linkage</t>
+  </si>
+  <si>
+    <t>STATIC categorical token</t>
+  </si>
+  <si>
+    <t>Trauma E-code workbook + diagnosis codes</t>
+  </si>
+  <si>
+    <t>Direct mapping to binary/3-class/2-class tokens.</t>
+  </si>
+  <si>
+    <t>Admission/diagnosis provenance should be preserved.</t>
+  </si>
+  <si>
+    <t>Use as static trauma mechanism with source provenance.</t>
+  </si>
+  <si>
+    <t>transfer</t>
+  </si>
+  <si>
+    <t>final_preicu_input</t>
+  </si>
+  <si>
+    <t>MIMIC-IV-ED arrival_transport plus admissions fallback</t>
+  </si>
+  <si>
+    <t>Map raw ED transport/admission source to transfer indicator/category.</t>
+  </si>
+  <si>
+    <t>Pre-ICU ED/admission information.</t>
+  </si>
+  <si>
+    <t>Requires ED linkage; fallback source should be tagged.</t>
+  </si>
+  <si>
+    <t>initial_ed_sbp</t>
+  </si>
+  <si>
+    <t>ED triage.sbp or first valid ED vitalsign SBP</t>
+  </si>
+  <si>
+    <t>Bucket: &lt;90→hypotension/90-110→borderline_low/&gt;=111→not_low. No numeric channel.</t>
+  </si>
+  <si>
+    <t>Pre-ICU ED measurement.</t>
+  </si>
+  <si>
+    <t>Requires ED linkage and physiologic filtering. NA if no ED.</t>
+  </si>
+  <si>
+    <t>rsi</t>
+  </si>
+  <si>
+    <t>ED SBP and ED HR</t>
+  </si>
+  <si>
+    <t>Bucket: &lt;=1.0→high_risk/1.1-1.7→intermediate/&gt;=1.8→low_risk. No numeric channel.</t>
+  </si>
+  <si>
+    <t>Pre-ICU ED measurement; requires both SBP and HR.</t>
+  </si>
+  <si>
+    <t>NA if no ED linkage or HR=0.</t>
+  </si>
+  <si>
+    <t>head_injury</t>
   </si>
   <si>
     <t>final_static_input</t>
   </si>
   <si>
-    <t>patients/admissions/cohort static fields</t>
-  </si>
-  <si>
-    <t>age = age_at_admit; male = 1 if gender == 'M' else 0.</t>
-  </si>
-  <si>
-    <t>Admission-known static fields.</t>
-  </si>
-  <si>
-    <t>No temporal leakage.</t>
-  </si>
-  <si>
-    <t>mechanism_cat</t>
-  </si>
-  <si>
-    <t>Trauma E-code workbook + diagnosis codes</t>
-  </si>
-  <si>
-    <t>Map to 1=blunt, 2=penetrating, 3=other_or_burn_or_unknown.</t>
-  </si>
-  <si>
-    <t>Admission/diagnosis provenance should be preserved.</t>
-  </si>
-  <si>
-    <t>Use as static trauma mechanism with source provenance.</t>
-  </si>
-  <si>
-    <t>transfer</t>
-  </si>
-  <si>
-    <t>final_preicu_input</t>
-  </si>
-  <si>
-    <t>MIMIC-IV-ED arrival_transport plus admissions fallback</t>
-  </si>
-  <si>
-    <t>Map raw ED transport/admission source to transfer indicator/category.</t>
-  </si>
-  <si>
-    <t>Pre-ICU ED/admission information.</t>
-  </si>
-  <si>
-    <t>Requires ED linkage; fallback source should be tagged.</t>
-  </si>
-  <si>
-    <t>initial_ed_sbp</t>
-  </si>
-  <si>
-    <t>ED triage.sbp or first valid ED vitalsign SBP</t>
-  </si>
-  <si>
-    <t>Use triage.sbp first; if missing, use first valid ED vitalsign SBP.</t>
-  </si>
-  <si>
-    <t>Pre-ICU ED measurement.</t>
-  </si>
-  <si>
-    <t>Requires ED linkage and physiologic filtering. NA if no ED.</t>
-  </si>
-  <si>
-    <t>rsi</t>
-  </si>
-  <si>
-    <t>ED SBP and ED HR</t>
-  </si>
-  <si>
-    <t>rSI = SBP / HR. Confirmed from uw_fields.png (Reverse Shock Index).</t>
-  </si>
-  <si>
-    <t>Pre-ICU ED measurement; requires both SBP and HR.</t>
-  </si>
-  <si>
-    <t>NA if no ED linkage or HR=0.</t>
-  </si>
-  <si>
-    <t>head_injury</t>
-  </si>
-  <si>
     <t>Hospital diagnosis ICD codes</t>
   </si>
   <si>
@@ -245,16 +257,16 @@
     <t>G2*</t>
   </si>
   <si>
-    <t>baseDef48 / lactate48 / RBC48 / crys48</t>
-  </si>
-  <si>
-    <t>conditional_daily_summary</t>
+    <t>base_def_48</t>
+  </si>
+  <si>
+    <t>DAY FIRST48 bucket</t>
   </si>
   <si>
     <t>base_excess / lactate / RBC inputevents / crystalloid inputevents</t>
   </si>
   <si>
-    <t>Aggregate over completed first 48h window. Appears in daily block only when history &gt;= 48h.</t>
+    <t>base_deficit=max(0,-base_excess). Bucket: mild/moderate/severe. Once at source_day_index=1.</t>
   </si>
   <si>
     <t>May appear in daily/summary blocks only after completed summary coverage is &gt;=48h.</t>
@@ -266,16 +278,16 @@
     <t>G3</t>
   </si>
   <si>
-    <t>bolusSum_h / RBCsum_h</t>
-  </si>
-  <si>
-    <t>final_derived_input</t>
+    <t>RBCsum</t>
+  </si>
+  <si>
+    <t>DAY event token</t>
   </si>
   <si>
     <t>iv_fluid_ml_1h / rbc_ml_1h implementation variables</t>
   </si>
   <si>
-    <t>bolusSum_h = sum_{tau &lt;= h}(iv_fluid_ml_1h_tau); RBCsum_h = sum_{tau &lt;= h}(rbc_ml_1h_tau).</t>
+    <t>Any RBC&gt;0→[rbc_transfusion_event_present]. Moved from HOUR.</t>
   </si>
   <si>
     <t>Use only fluid/RBC events delivered at or before h.</t>
@@ -287,16 +299,16 @@
     <t>VENT</t>
   </si>
   <si>
-    <t>vent_h / ventDaySum_h</t>
-  </si>
-  <si>
-    <t>final_hourly_status / emphasis flag</t>
+    <t>vent_h</t>
+  </si>
+  <si>
+    <t>HOUR sparse event token</t>
   </si>
   <si>
     <t>ventilation status/procedure interval</t>
   </si>
   <si>
-    <t>vent_h = 1 if invasive ventilation active in hour h; ventDaySum_h = count distinct ICU days d &lt;= h with any vent=1.</t>
+    <t>[vent_on] when active. event_emb[vent_id]+hour_time_emb. After 7 vitals.</t>
   </si>
   <si>
     <t>Use only evidence available by h.</t>
@@ -305,13 +317,16 @@
     <t>Do not use future total ventilation at early landmarks.</t>
   </si>
   <si>
-    <t>surgHours_h / surgSum_h</t>
+    <t>surgHours/surgSum</t>
+  </si>
+  <si>
+    <t>DAY event token source</t>
   </si>
   <si>
     <t>surgery_hours_1h implementation variable</t>
   </si>
   <si>
-    <t>surgHours_h = sum_{tau &lt;= h}(surgery_hours_1h_tau); surgSum_h = count distinct ICU days with surgery.</t>
+    <t>Delta&gt;0→[surgery_in_window].</t>
   </si>
   <si>
     <t>Use OR overlap up to h only.</t>
@@ -323,16 +338,16 @@
     <t>G4</t>
   </si>
   <si>
-    <t>bicarb / bun / creatinine / wbc / lymphocytes / neutrophils</t>
-  </si>
-  <si>
-    <t>final_lab_memory_input</t>
+    <t>bicarb</t>
+  </si>
+  <si>
+    <t>DAY bucket</t>
   </si>
   <si>
     <t>labevents</t>
   </si>
   <si>
-    <t>latest_value_at_or_before_h + observed_h + time_since_last_h.</t>
+    <t>Min&lt;22→[bicarbonate_min_bin_low].</t>
   </si>
   <si>
     <t>Use only lab observations at or before h.</t>
@@ -341,16 +356,16 @@
     <t>Do not use future labs.</t>
   </si>
   <si>
-    <t>uop_h</t>
-  </si>
-  <si>
-    <t>final_hourly_output</t>
+    <t>uop</t>
+  </si>
+  <si>
+    <t>DAY data quality</t>
   </si>
   <si>
     <t>outputevents urine itemids</t>
   </si>
   <si>
-    <t>uop_h = sum(urine output volume overlapping hour h).</t>
+    <t>Measured hours: &gt;=6→measured/1-5→sparse/0→not_measured.</t>
   </si>
   <si>
     <t>Use output event time/interval at or before h.</t>
@@ -359,22 +374,115 @@
     <t>Interval splitting must be leakage-safe.</t>
   </si>
   <si>
-    <t>StrongIon_h</t>
-  </si>
-  <si>
-    <t>final_derived_lab_memory</t>
+    <t>StrongIon</t>
+  </si>
+  <si>
+    <t>Hold</t>
   </si>
   <si>
     <t>Na_h, K_h, Cl_h, bicarb_h</t>
   </si>
   <si>
-    <t>StrongIon = (Na + K) - (Cl + bicarb).</t>
+    <t>Hold. No frozen gate.</t>
   </si>
   <si>
     <t>Use latest aligned values at or before h.</t>
   </si>
   <si>
     <t>Na/K/Cl are intermediate variables.</t>
+  </si>
+  <si>
+    <t>surg48</t>
+  </si>
+  <si>
+    <t>procedureevents OR procedures</t>
+  </si>
+  <si>
+    <t>Count OR procedures. Bucket: 1/2/3+. 0=silent. Once.</t>
+  </si>
+  <si>
+    <t>Only when &gt;=48h history.</t>
+  </si>
+  <si>
+    <t>Not emitted if &lt;48h.</t>
+  </si>
+  <si>
+    <t>abx48</t>
+  </si>
+  <si>
+    <t>prescriptions antibiotic</t>
+  </si>
+  <si>
+    <t>Any antibiotic→[antibiotics_in_window].</t>
+  </si>
+  <si>
+    <t>Per DAY window.</t>
+  </si>
+  <si>
+    <t>No leakage.</t>
+  </si>
+  <si>
+    <t>CXR</t>
+  </si>
+  <si>
+    <t>cxr_finding</t>
+  </si>
+  <si>
+    <t>CXR event token</t>
+  </si>
+  <si>
+    <t>MIMIC-CXR-JPG CheXpert CSV</t>
+  </si>
+  <si>
+    <t>12 findings. Positive→[cxr_finding_*].</t>
+  </si>
+  <si>
+    <t>Only studies with datetime &lt;= t.</t>
+  </si>
+  <si>
+    <t>No future CXR.</t>
+  </si>
+  <si>
+    <t>DQ</t>
+  </si>
+  <si>
+    <t>core_vital_slots</t>
+  </si>
+  <si>
+    <t>chartevents hr,sbp,dbp,map,rr,temp</t>
+  </si>
+  <si>
+    <t>Observed/eligible. Denom=wh*6. &gt;=83%→dense/50-82%→partial/1-49%→sparse/0→none.</t>
+  </si>
+  <si>
+    <t>FiO2 excluded.</t>
+  </si>
+  <si>
+    <t>lab_draw_status</t>
+  </si>
+  <si>
+    <t>labevents bicarb,bun,creatinine,wbc</t>
+  </si>
+  <si>
+    <t>0 draws→[labs_not_drawn]; &gt;=1→silent.</t>
+  </si>
+  <si>
+    <t>No future labs.</t>
+  </si>
+  <si>
+    <t>day_window_len</t>
+  </si>
+  <si>
+    <t>DAY structural token</t>
+  </si>
+  <si>
+    <t>ICU day boundaries</t>
+  </si>
+  <si>
+    <t>24 tokens: [day_window_len_01h]...[day_window_len_24h].</t>
+  </si>
+  <si>
+    <t>Per DAY block.</t>
   </si>
   <si>
     <t>meaning</t>
@@ -407,8 +515,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -425,7 +533,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -474,6 +582,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -502,7 +616,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -528,12 +642,24 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -821,20 +947,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G20"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G26"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.7109375" customWidth="1"/>
-    <col min="2" max="2" width="38.7109375" customWidth="1"/>
-    <col min="3" max="3" width="26.7109375" customWidth="1"/>
-    <col min="4" max="4" width="46.7109375" customWidth="1"/>
-    <col min="5" max="5" width="78.7109375" customWidth="1"/>
-    <col min="6" max="6" width="50.7109375" customWidth="1"/>
-    <col min="7" max="7" width="52.7109375" customWidth="1"/>
+    <col min="1" max="1" width="10.7265625" customWidth="1"/>
+    <col min="2" max="2" width="38.7265625" customWidth="1"/>
+    <col min="3" max="3" width="26.7265625" customWidth="1"/>
+    <col min="4" max="4" width="46.7265625" customWidth="1"/>
+    <col min="5" max="5" width="78.7265625" customWidth="1"/>
+    <col min="6" max="6" width="50.7265625" customWidth="1"/>
+    <col min="7" max="7" width="52.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -857,7 +983,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
@@ -880,7 +1006,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>7</v>
       </c>
@@ -903,7 +1029,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
@@ -926,7 +1052,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>22</v>
       </c>
@@ -949,7 +1075,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
         <v>29</v>
       </c>
@@ -972,7 +1098,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
         <v>29</v>
       </c>
@@ -980,397 +1106,535 @@
         <v>36</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
         <v>29</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
         <v>29</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
         <v>29</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="s">
         <v>29</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>31</v>
+        <v>59</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
         <v>29</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="4" t="s">
         <v>29</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C14" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A15" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="F16" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="G16" s="9" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A17" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A18" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A19" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="G19" s="7" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A20" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
         <v>76</v>
       </c>
-      <c r="D14" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="E14" s="5" t="s">
+      <c r="B21" t="s">
+        <v>122</v>
+      </c>
+      <c r="C21" t="s">
         <v>78</v>
       </c>
-      <c r="F14" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="G14" s="5" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7">
-      <c r="A15" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="C15" s="6" t="s">
+      <c r="D21" t="s">
+        <v>123</v>
+      </c>
+      <c r="E21" t="s">
+        <v>124</v>
+      </c>
+      <c r="F21" t="s">
+        <v>125</v>
+      </c>
+      <c r="G21" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
         <v>83</v>
       </c>
-      <c r="D15" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="E15" s="6" t="s">
+      <c r="B22" t="s">
+        <v>127</v>
+      </c>
+      <c r="C22" t="s">
         <v>85</v>
       </c>
-      <c r="F15" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="G15" s="6" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7">
-      <c r="A16" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7">
-      <c r="A17" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="E17" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="F17" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="G17" s="6" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7">
-      <c r="A18" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="B18" s="7" t="s">
-        <v>101</v>
-      </c>
-      <c r="C18" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="D18" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="E18" s="7" t="s">
-        <v>104</v>
-      </c>
-      <c r="F18" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="G18" s="7" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7">
-      <c r="A19" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="B19" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="C19" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="D19" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="E19" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="F19" s="7" t="s">
+      <c r="D22" t="s">
+        <v>128</v>
+      </c>
+      <c r="E22" t="s">
+        <v>129</v>
+      </c>
+      <c r="F22" t="s">
+        <v>130</v>
+      </c>
+      <c r="G22" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>132</v>
+      </c>
+      <c r="B23" t="s">
+        <v>133</v>
+      </c>
+      <c r="C23" t="s">
+        <v>134</v>
+      </c>
+      <c r="D23" t="s">
+        <v>135</v>
+      </c>
+      <c r="E23" t="s">
+        <v>136</v>
+      </c>
+      <c r="F23" t="s">
+        <v>137</v>
+      </c>
+      <c r="G23" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>139</v>
+      </c>
+      <c r="B24" t="s">
+        <v>140</v>
+      </c>
+      <c r="C24" t="s">
         <v>111</v>
       </c>
-      <c r="G19" s="7" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7">
-      <c r="A20" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="B20" s="7" t="s">
-        <v>113</v>
-      </c>
-      <c r="C20" s="7" t="s">
-        <v>114</v>
-      </c>
-      <c r="D20" s="7" t="s">
-        <v>115</v>
-      </c>
-      <c r="E20" s="7" t="s">
-        <v>116</v>
-      </c>
-      <c r="F20" s="7" t="s">
-        <v>117</v>
-      </c>
-      <c r="G20" s="7" t="s">
-        <v>118</v>
+      <c r="D24" t="s">
+        <v>141</v>
+      </c>
+      <c r="E24" t="s">
+        <v>142</v>
+      </c>
+      <c r="F24" t="s">
+        <v>130</v>
+      </c>
+      <c r="G24" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>139</v>
+      </c>
+      <c r="B25" t="s">
+        <v>144</v>
+      </c>
+      <c r="C25" t="s">
+        <v>111</v>
+      </c>
+      <c r="D25" t="s">
+        <v>145</v>
+      </c>
+      <c r="E25" t="s">
+        <v>146</v>
+      </c>
+      <c r="F25" t="s">
+        <v>130</v>
+      </c>
+      <c r="G25" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>139</v>
+      </c>
+      <c r="B26" t="s">
+        <v>148</v>
+      </c>
+      <c r="C26" t="s">
+        <v>149</v>
+      </c>
+      <c r="D26" t="s">
+        <v>150</v>
+      </c>
+      <c r="E26" t="s">
+        <v>151</v>
+      </c>
+      <c r="F26" t="s">
+        <v>152</v>
+      </c>
+      <c r="G26" t="s">
+        <v>131</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G20"/>
+  <autoFilter ref="A1:G20" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.7109375" customWidth="1"/>
-    <col min="2" max="2" width="72.7109375" customWidth="1"/>
+    <col min="1" max="1" width="16.7265625" customWidth="1"/>
+    <col min="2" max="2" width="72.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
         <v>29</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" s="7" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" s="8" t="s">
-        <v>126</v>
+        <v>160</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>127</v>
+        <v>161</v>
       </c>
     </row>
   </sheetData>

</xml_diff>